<commit_message>
QC pass: fix Semester 1 lesson gaps and MCQ answer bias
Lessons (Units 1-13): close small forward-reference and undocumented-
builtin gaps found during a full sequencing review (round(), .isdigit()/
.isalpha(), premature comparison-operator use, list/dict truthiness
preview, datetime.strptime, uv lesson framing), and remove 14 orphaned
image files from Unit 2 that no lesson referenced.

MCQ bank (all 13 units, 40 questions each): the correct answer was the
uniquely longest option far more often than chance (27.5%-85% per unit,
vs. a 25% baseline), letting a "pick the longest" heuristic beat the
quiz. Rewrote the under-written distractor on every flagged question to
close the gap, and reshuffled option order per question so each unit's
answer key lands at a balanced ~12/12/8/8 split across positions A-D
instead of a skewed or repetitive pattern.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/content/Question Bank/MCQ/Unit 1 - Introduction to Programming/Unit 1 - Introduction to Programming - MCQ.xlsx
+++ b/content/Question Bank/MCQ/Unit 1 - Introduction to Programming/Unit 1 - Introduction to Programming - MCQ.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Python - MCQ - 1.1" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Python - MCQ - 1.2" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Python - MCQ - 1.3" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Python - MCQ - 1.4" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Python - MCQ - 1.1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Python - MCQ - 1.2" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Python - MCQ - 1.3" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Python - MCQ - 1.4" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -643,26 +643,26 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
+          <t>The loop stops immediately and total simply becomes 5</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>It produces a syntax error before running</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
           <t>The loop runs forever because i is never updated</t>
         </is>
       </c>
-      <c r="N2" t="inlineStr">
+      <c r="P2" t="inlineStr">
         <is>
           <t>It runs correctly and total ends up being 15</t>
         </is>
       </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>The loop stops immediately and total simply becomes 5</t>
-        </is>
-      </c>
-      <c r="P2" t="inlineStr">
-        <is>
-          <t>It produces a syntax error before running</t>
-        </is>
-      </c>
       <c r="Q2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3">
@@ -726,17 +726,17 @@
       </c>
       <c r="N3" t="inlineStr">
         <is>
+          <t>Look back: reviewing the solution only after it is delivered</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
           <t>Plan: jumping to choosing a coding structure too early</t>
         </is>
       </c>
-      <c r="O3" t="inlineStr">
+      <c r="P3" t="inlineStr">
         <is>
           <t>Carry out: writing the implementation code directly</t>
-        </is>
-      </c>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t>Look back: reviewing the solution only after it is delivered</t>
         </is>
       </c>
       <c r="Q3" t="n">
@@ -799,26 +799,26 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
+          <t>`False`, because computers cannot process any human language at all, spoken or written</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
           <t>`False`, even sophisticated systems run on precisely specified instructions; nothing is inferred unless explicitly programmed</t>
         </is>
       </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>`False`, because computers cannot process any human language at all, spoken or written</t>
-        </is>
-      </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>`True`, computers can infer any vague instruction once they have been trained on enough examples</t>
+          <t>`True`, but only for advanced artificial intelligence programs that mimic human reasoning</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>`True`, but only for advanced artificial intelligence programs that mimic human reasoning</t>
+          <t>`True`, computers can infer any vague instruction once they have been trained on enough real-world examples and context</t>
         </is>
       </c>
       <c r="Q4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="5">
@@ -877,26 +877,26 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
+          <t>Output stage</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>Storage stage</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>Input stage</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
           <t>Processing stage</t>
         </is>
       </c>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>Storage stage</t>
-        </is>
-      </c>
-      <c r="O5" t="inlineStr">
-        <is>
-          <t>Output stage</t>
-        </is>
-      </c>
-      <c r="P5" t="inlineStr">
-        <is>
-          <t>Input stage</t>
-        </is>
-      </c>
       <c r="Q5" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6">
@@ -960,21 +960,21 @@
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>Code typed directly in the REPL is automatically and permanently saved for reuse</t>
+          <t>A .py script can be saved and run again, while the REPL is best for quick, throwaway experiments</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
         <is>
+          <t>Code typed directly in the REPL is automatically and permanently saved for later reuse</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
           <t>The REPL interprets a completely different programming language than scripts do</t>
         </is>
       </c>
-      <c r="P6" t="inlineStr">
-        <is>
-          <t>A .py script can be saved and run again, while the REPL is best for quick, throwaway experiments</t>
-        </is>
-      </c>
       <c r="Q6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="7">
@@ -1033,26 +1033,26 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
+          <t>Pattern recognition</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>Debugging</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>Decomposition</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
           <t>Abstraction</t>
         </is>
       </c>
-      <c r="N7" t="inlineStr">
-        <is>
-          <t>Debugging</t>
-        </is>
-      </c>
-      <c r="O7" t="inlineStr">
-        <is>
-          <t>Decomposition</t>
-        </is>
-      </c>
-      <c r="P7" t="inlineStr">
-        <is>
-          <t>Pattern recognition</t>
-        </is>
-      </c>
       <c r="Q7" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="8">
@@ -1111,7 +1111,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>It translates the source code directly into low-level hardware signals</t>
+          <t>Code is read and executed line by line by the interpreter, with no separate compile step</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
@@ -1121,7 +1121,7 @@
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>Code is read and executed line by line by the interpreter, with no separate compile step</t>
+          <t>It translates source code directly into hardware signals, no interpreter needed</t>
         </is>
       </c>
       <c r="P8" t="inlineStr">
@@ -1130,7 +1130,7 @@
         </is>
       </c>
       <c r="Q8" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9">
@@ -1194,17 +1194,17 @@
       </c>
       <c r="N9" t="inlineStr">
         <is>
+          <t>Rectangle</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
           <t>Parallelogram</t>
         </is>
       </c>
-      <c r="O9" t="inlineStr">
+      <c r="P9" t="inlineStr">
         <is>
           <t>Oval</t>
-        </is>
-      </c>
-      <c r="P9" t="inlineStr">
-        <is>
-          <t>Rectangle</t>
         </is>
       </c>
       <c r="Q9" t="n">
@@ -1267,22 +1267,22 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
+          <t>Decomposition</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>Compilation</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>Abstraction</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
           <t>Pattern recognition</t>
-        </is>
-      </c>
-      <c r="N10" t="inlineStr">
-        <is>
-          <t>Compilation</t>
-        </is>
-      </c>
-      <c r="O10" t="inlineStr">
-        <is>
-          <t>Decomposition</t>
-        </is>
-      </c>
-      <c r="P10" t="inlineStr">
-        <is>
-          <t>Abstraction</t>
         </is>
       </c>
       <c r="Q10" t="n">
@@ -1345,26 +1345,26 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
+          <t>A random, unordered collection of instructions with no clear goal</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
           <t>A specific programming language used to write software</t>
         </is>
       </c>
-      <c r="N11" t="inlineStr">
+      <c r="O11" t="inlineStr">
         <is>
           <t>A finite, ordered set of clear, unambiguous steps that solves a problem</t>
         </is>
       </c>
-      <c r="O11" t="inlineStr">
-        <is>
-          <t>A random, unordered collection of instructions with no clear goal</t>
-        </is>
-      </c>
       <c r="P11" t="inlineStr">
         <is>
           <t>A physical type of computer hardware component</t>
         </is>
       </c>
       <c r="Q11" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
   </sheetData>
@@ -1524,26 +1524,26 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
+          <t>Designing the physical layout of a circuit board</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
           <t>Repairing computer hardware components when they physically malfunction</t>
         </is>
       </c>
-      <c r="N2" t="inlineStr">
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>Using existing applications such as a web browser or word processor</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
         <is>
           <t>Giving a computer a clear, ordered set of instructions to perform a task</t>
         </is>
       </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>Designing the physical layout of a circuit board</t>
-        </is>
-      </c>
-      <c r="P2" t="inlineStr">
-        <is>
-          <t>Using existing applications such as a web browser or word processor</t>
-        </is>
-      </c>
       <c r="Q2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3">
@@ -1602,26 +1602,26 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
+          <t>Carry out, Plan, Understand, Look back</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
           <t>Understand, Carry out, Plan, Look back</t>
         </is>
       </c>
-      <c r="N3" t="inlineStr">
+      <c r="O3" t="inlineStr">
         <is>
           <t>Understand, Plan, Carry out, Look back</t>
         </is>
       </c>
-      <c r="O3" t="inlineStr">
+      <c r="P3" t="inlineStr">
         <is>
           <t>Plan, Understand, Look back, Carry out</t>
         </is>
       </c>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t>Carry out, Plan, Understand, Look back</t>
-        </is>
-      </c>
       <c r="Q3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="4">
@@ -1685,17 +1685,17 @@
       </c>
       <c r="N4" t="inlineStr">
         <is>
+          <t>Well-designed programs should always rely on loops to work correctly</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
           <t>Computers can automatically infer any missing steps on their own</t>
         </is>
       </c>
-      <c r="O4" t="inlineStr">
-        <is>
-          <t>Well-designed programs should always rely on loops to work correctly</t>
-        </is>
-      </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>Real-world tasks like this can never be represented accurately in code</t>
+          <t>Real-world tasks like this can never be represented accurately in programming code</t>
         </is>
       </c>
       <c r="Q4" t="n">
@@ -1763,21 +1763,21 @@
       </c>
       <c r="N5" t="inlineStr">
         <is>
+          <t>Input, Processing, Output</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>Input, Print, Output</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
           <t>Initialize, Process, Order</t>
         </is>
       </c>
-      <c r="O5" t="inlineStr">
-        <is>
-          <t>Input, Print, Output</t>
-        </is>
-      </c>
-      <c r="P5" t="inlineStr">
-        <is>
-          <t>Input, Processing, Output</t>
-        </is>
-      </c>
       <c r="Q5" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="6">
@@ -1841,17 +1841,17 @@
       </c>
       <c r="N6" t="inlineStr">
         <is>
+          <t>Abstraction is incorrectly hiding important sensor implementation details</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>Pattern recognition has failed to spot the repeating structure</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
           <t>The algorithm fails the finiteness requirement of a proper algorithm</t>
-        </is>
-      </c>
-      <c r="O6" t="inlineStr">
-        <is>
-          <t>Pattern recognition has failed to spot the repeating structure</t>
-        </is>
-      </c>
-      <c r="P6" t="inlineStr">
-        <is>
-          <t>Abstraction is incorrectly hiding important sensor implementation details</t>
         </is>
       </c>
       <c r="Q6" t="n">
@@ -1914,26 +1914,26 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>58</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
           <t>19</t>
         </is>
       </c>
-      <c r="N7" t="inlineStr">
-        <is>
-          <t>58</t>
-        </is>
-      </c>
-      <c r="O7" t="inlineStr">
-        <is>
-          <t>27</t>
-        </is>
-      </c>
       <c r="P7" t="inlineStr">
         <is>
           <t>12</t>
         </is>
       </c>
       <c r="Q7" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8">
@@ -1992,22 +1992,22 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
+          <t>An error</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>Hello, World!</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>Hello, World! (including the quotes)</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
           <t>Nothing</t>
-        </is>
-      </c>
-      <c r="N8" t="inlineStr">
-        <is>
-          <t>Hello, World!</t>
-        </is>
-      </c>
-      <c r="O8" t="inlineStr">
-        <is>
-          <t>Hello, World! (including the quotes)</t>
-        </is>
-      </c>
-      <c r="P8" t="inlineStr">
-        <is>
-          <t>An error</t>
         </is>
       </c>
       <c r="Q8" t="n">
@@ -2070,26 +2070,26 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
+          <t>Iteration</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>Decomposition</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>Pattern recognition</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
           <t>Abstraction</t>
         </is>
       </c>
-      <c r="N9" t="inlineStr">
-        <is>
-          <t>Pattern recognition</t>
-        </is>
-      </c>
-      <c r="O9" t="inlineStr">
-        <is>
-          <t>Decomposition</t>
-        </is>
-      </c>
-      <c r="P9" t="inlineStr">
-        <is>
-          <t>Iteration</t>
-        </is>
-      </c>
       <c r="Q9" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="10">
@@ -2158,16 +2158,16 @@
       </c>
       <c r="O10" t="inlineStr">
         <is>
+          <t>Start writing code immediately without a plan</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
           <t>Understand the problem (inputs, outputs, constraints)</t>
         </is>
       </c>
-      <c r="P10" t="inlineStr">
-        <is>
-          <t>Start writing code immediately without a plan</t>
-        </is>
-      </c>
       <c r="Q10" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="11">
@@ -2226,26 +2226,26 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
           <t>4</t>
         </is>
       </c>
-      <c r="N11" t="inlineStr">
+      <c r="O11" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="O11" t="inlineStr">
-        <is>
-          <t>24</t>
-        </is>
-      </c>
       <c r="P11" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
       <c r="Q11" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
   </sheetData>
@@ -2410,21 +2410,21 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
+          <t>Python programs always run faster than any compiled language</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
           <t>Slightly slower raw execution speed in exchange for faster, simpler development and testing</t>
         </is>
       </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>Python programs always run faster than any compiled language</t>
-        </is>
-      </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>Python code cannot be tested at all until the entire program is finished</t>
+          <t>Python code cannot be tested at all until the entire program has been completely finished</t>
         </is>
       </c>
       <c r="Q2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3">
@@ -2483,26 +2483,26 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
+          <t>Oval (start/end terminator)</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>Parallelogram (input/output)</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
           <t>Circle (used for connectors)</t>
         </is>
       </c>
-      <c r="N3" t="inlineStr">
+      <c r="P3" t="inlineStr">
         <is>
           <t>Diamond (decision)</t>
         </is>
       </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>Parallelogram (input/output)</t>
-        </is>
-      </c>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t>Oval (start/end terminator)</t>
-        </is>
-      </c>
       <c r="Q3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4">
@@ -2566,21 +2566,21 @@
       </c>
       <c r="N4" t="inlineStr">
         <is>
+          <t>Exactly and in order, without assuming intent</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>By guessing what you most likely wanted</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
           <t>By choosing the fastest result regardless of order</t>
         </is>
       </c>
-      <c r="O4" t="inlineStr">
-        <is>
-          <t>By guessing what you most likely wanted</t>
-        </is>
-      </c>
-      <c r="P4" t="inlineStr">
-        <is>
-          <t>Exactly and in order, without assuming intent</t>
-        </is>
-      </c>
       <c r="Q4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="5">
@@ -2639,26 +2639,26 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
+          <t>Garbage in, garbage out: output quality depends on input quality</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>Abstraction: hiding implementation detail behind an interface</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>Syntax error: code that breaks Python's grammar rules</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
           <t>Infinite loop: a loop condition that never becomes false</t>
         </is>
       </c>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>Garbage in, garbage out: output quality depends on input quality</t>
-        </is>
-      </c>
-      <c r="O5" t="inlineStr">
-        <is>
-          <t>Syntax error: code that breaks Python's grammar rules</t>
-        </is>
-      </c>
-      <c r="P5" t="inlineStr">
-        <is>
-          <t>Abstraction: hiding implementation detail behind an interface</t>
-        </is>
-      </c>
       <c r="Q5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6">
@@ -2717,12 +2717,12 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
+          <t>Definiteness</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
           <t>Output</t>
-        </is>
-      </c>
-      <c r="N6" t="inlineStr">
-        <is>
-          <t>Definiteness</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
@@ -2800,17 +2800,17 @@
       </c>
       <c r="N7" t="inlineStr">
         <is>
+          <t>Compare each pair and swap if out of order</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>Add 2 to the number</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
           <t>Print the result</t>
-        </is>
-      </c>
-      <c r="O7" t="inlineStr">
-        <is>
-          <t>Add 2 to the number</t>
-        </is>
-      </c>
-      <c r="P7" t="inlineStr">
-        <is>
-          <t>Compare each pair and swap if out of order</t>
         </is>
       </c>
       <c r="Q7" t="n">
@@ -2878,21 +2878,21 @@
       </c>
       <c r="N8" t="inlineStr">
         <is>
+          <t>.exe</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
           <t>.py</t>
         </is>
       </c>
-      <c r="O8" t="inlineStr">
+      <c r="P8" t="inlineStr">
         <is>
           <t>.pyt</t>
         </is>
       </c>
-      <c r="P8" t="inlineStr">
-        <is>
-          <t>.exe</t>
-        </is>
-      </c>
       <c r="Q8" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="9">
@@ -2951,12 +2951,12 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
+          <t>It is functionally identical to raw machine code</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
           <t>It must follow Python's exact syntax rules precisely</t>
-        </is>
-      </c>
-      <c r="N9" t="inlineStr">
-        <is>
-          <t>It is functionally identical to raw machine code</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
@@ -3029,26 +3029,26 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
+          <t>A built-in tool that monitors a laptop's battery charge level</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
           <t>A large standard library plus many third-party packages, so you rarely build from scratch</t>
         </is>
       </c>
-      <c r="N10" t="inlineStr">
-        <is>
-          <t>A limitation in Python that actively prevents installing any packages</t>
-        </is>
-      </c>
       <c r="O10" t="inlineStr">
         <is>
+          <t>A limitation in Python that actively prevents installing any third-party packages</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
           <t>A quirky claim that Python needs actual physical batteries to run</t>
         </is>
       </c>
-      <c r="P10" t="inlineStr">
-        <is>
-          <t>A built-in tool that monitors a laptop's battery charge level</t>
-        </is>
-      </c>
       <c r="Q10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="11">
@@ -3107,26 +3107,26 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
+          <t>Oval (terminator)</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
           <t>Rectangle (process)</t>
         </is>
       </c>
-      <c r="N11" t="inlineStr">
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>Diamond (decision)</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
         <is>
           <t>Arrow (flow line)</t>
         </is>
       </c>
-      <c r="O11" t="inlineStr">
-        <is>
-          <t>Diamond (decision)</t>
-        </is>
-      </c>
-      <c r="P11" t="inlineStr">
-        <is>
-          <t>Oval (terminator)</t>
-        </is>
-      </c>
       <c r="Q11" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -3286,26 +3286,26 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
+          <t>A program and a programming language mean exactly the same thing</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>Program = computer hardware; Language = the operating system</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
           <t>Program = a set of instructions that performs a task; Language = the medium used to write it</t>
         </is>
       </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>A program and a programming language mean exactly the same thing</t>
-        </is>
-      </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>Program = computer hardware; Language = the operating system</t>
-        </is>
-      </c>
       <c r="P2" t="inlineStr">
         <is>
           <t>Program = a language the computer understands; Language = a saved set of instructions</t>
         </is>
       </c>
       <c r="Q2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3">
@@ -3364,26 +3364,26 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
+          <t>Printing the payslip</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
           <t>Calculating the pay</t>
         </is>
       </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>Printing the payslip</t>
-        </is>
-      </c>
       <c r="O3" t="inlineStr">
         <is>
+          <t>Storing the employee ID</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
           <t>Reading the hours worked</t>
         </is>
       </c>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t>Storing the employee ID</t>
-        </is>
-      </c>
       <c r="Q3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4">
@@ -3442,26 +3442,26 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
+          <t>It violates input because no input is taken</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
           <t>It violates definiteness because the steps are ambiguous</t>
         </is>
       </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>It violates input because no input is taken</t>
-        </is>
-      </c>
       <c r="O4" t="inlineStr">
         <is>
+          <t>It is valid; algorithms are allowed to run forever</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
           <t>It violates finiteness because the loop never terminates</t>
         </is>
       </c>
-      <c r="P4" t="inlineStr">
-        <is>
-          <t>It is valid; algorithms are allowed to run forever</t>
-        </is>
-      </c>
       <c r="Q4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="5">
@@ -3520,26 +3520,26 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
+          <t>Line (c)</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>Line (b)</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
           <t>Line (a)</t>
         </is>
       </c>
-      <c r="N5" t="inlineStr">
+      <c r="P5" t="inlineStr">
         <is>
           <t>Line (d)</t>
         </is>
       </c>
-      <c r="O5" t="inlineStr">
-        <is>
-          <t>Line (c)</t>
-        </is>
-      </c>
-      <c r="P5" t="inlineStr">
-        <is>
-          <t>Line (b)</t>
-        </is>
-      </c>
       <c r="Q5" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="6">
@@ -3598,26 +3598,26 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
+          <t>Python parses the whole script first; a syntax error stops it from running at all</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>The REPL alone would have caught this mistake, but a saved script never would</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
           <t>Missing commas are only warnings in Python, never real errors</t>
         </is>
       </c>
-      <c r="N6" t="inlineStr">
-        <is>
-          <t>Python parses the whole script first; a syntax error stops it from running at all</t>
-        </is>
-      </c>
-      <c r="O6" t="inlineStr">
-        <is>
-          <t>The REPL alone would have caught this mistake, but a saved script never would</t>
-        </is>
-      </c>
       <c r="P6" t="inlineStr">
         <is>
           <t>Python ran the first working half of the script before it eventually crashed</t>
         </is>
       </c>
       <c r="Q6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7">
@@ -3676,22 +3676,22 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
+          <t>Data abstraction</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>Pattern recognition</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
           <t>Compilation step</t>
         </is>
       </c>
-      <c r="N7" t="inlineStr">
-        <is>
-          <t>Pattern recognition</t>
-        </is>
-      </c>
-      <c r="O7" t="inlineStr">
+      <c r="P7" t="inlineStr">
         <is>
           <t>Input validation</t>
-        </is>
-      </c>
-      <c r="P7" t="inlineStr">
-        <is>
-          <t>Data abstraction</t>
         </is>
       </c>
       <c r="Q7" t="n">
@@ -3754,26 +3754,26 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
+          <t>Look back (review): verifying edge and boundary cases</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
           <t>Plan: choosing an approach before writing any code</t>
         </is>
       </c>
-      <c r="N8" t="inlineStr">
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>Understand: restating the problem in your own words</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
         <is>
           <t>Carry out: typing the code needed for the solution</t>
         </is>
       </c>
-      <c r="O8" t="inlineStr">
-        <is>
-          <t>Look back (review): verifying edge and boundary cases</t>
-        </is>
-      </c>
-      <c r="P8" t="inlineStr">
-        <is>
-          <t>Understand: restating the problem in your own words</t>
-        </is>
-      </c>
       <c r="Q8" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9">
@@ -3832,26 +3832,26 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
+          <t>Completely replace the need for later testing</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
           <t>Compile and run noticeably faster than real Python code</t>
         </is>
       </c>
-      <c r="N9" t="inlineStr">
-        <is>
-          <t>Completely replace the need for later testing</t>
-        </is>
-      </c>
       <c r="O9" t="inlineStr">
         <is>
+          <t>Run directly on a computer without any translation</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
           <t>Describe an algorithm's logic in a readable, language-independent way</t>
         </is>
       </c>
-      <c r="P9" t="inlineStr">
-        <is>
-          <t>Run directly on a computer without any translation</t>
-        </is>
-      </c>
       <c r="Q9" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="10">
@@ -3910,14 +3910,14 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
+          <t>A specialised hardware description language</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
           <t>High-level, interpreted, general-purpose language</t>
         </is>
       </c>
-      <c r="N10" t="inlineStr">
-        <is>
-          <t>A specialised hardware description language</t>
-        </is>
-      </c>
       <c r="O10" t="inlineStr">
         <is>
           <t>A strictly low-level, fully compiled language</t>
@@ -3929,7 +3929,7 @@
         </is>
       </c>
       <c r="Q10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="11">
@@ -3993,17 +3993,17 @@
       </c>
       <c r="N11" t="inlineStr">
         <is>
+          <t>Oval (terminator)</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>Rectangle (process)</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
           <t>Diamond (decision)</t>
-        </is>
-      </c>
-      <c r="O11" t="inlineStr">
-        <is>
-          <t>Rectangle (process)</t>
-        </is>
-      </c>
-      <c r="P11" t="inlineStr">
-        <is>
-          <t>Oval (terminator)</t>
         </is>
       </c>
       <c r="Q11" t="n">

</xml_diff>